<commit_message>
Add TMA logo, fix Configure Display, add AI Assistant, enhance seed data
- Replace Plane icon with TMA logo SVG in sidebar and header
- Fix Configure Display: update contract DEFAULT_COLUMNS to match accordion
  structure, make ContractTable render columns dynamically from settings,
  remove stale "destinations" reference from TableSettingsModal
- Add AI Assistant module with Ollama integration: streaming chat interface,
  contract data context injection, connection status, model selection,
  suggestion prompts, and disconnected state with setup instructions
- Enhance seed data: 19 sub-contracts across 10 parent contracts with
  multiple sub-contracts per parent (1-3), mixed statuses (active/expiring/
  expired), 1-3 year durations, varied pricing ($320-$950), and comprehensive
  parameter data for all sub-contracts

https://claude.ai/code/session_01Ns76Dk5jS7GCzcCgigKWQ7
</commit_message>
<xml_diff>
--- a/public/data/atolls.xlsx
+++ b/public/data/atolls.xlsx
@@ -415,13 +415,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>bf15b042-aaa6-4622-be5e-116c34436d9b</v>
+        <v>c983362a-e407-41dc-ad5b-66e7bc09cc4b</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D2" t="str">
         <v>North Malé Atoll</v>
@@ -429,13 +429,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>03bb07fa-af5a-47c3-81e9-4b8e5a4c21c4</v>
+        <v>78ce8bc7-a017-426c-98a4-3031ce36ceca</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D3" t="str">
         <v>South Malé Atoll</v>
@@ -443,13 +443,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>e5443f5b-a3ff-4db6-b22c-aee5ee023fcd</v>
+        <v>0cf24454-7cc9-42b9-a277-594cd7494cbe</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D4" t="str">
         <v>Baa Atoll</v>
@@ -457,13 +457,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>35fc9789-3947-4c60-ba17-be8fdb63ecb8</v>
+        <v>cd2b459a-a775-4a2a-8c9f-331b1a16acc5</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D5" t="str">
         <v>Noonu Atoll</v>
@@ -471,13 +471,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>b47fb657-536f-4aff-966b-959da6866c24</v>
+        <v>efe70fbd-71d6-419c-9ebe-8d0ab0710f32</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D6" t="str">
         <v>Dhaalu Atoll</v>
@@ -485,13 +485,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>6e1ad3e3-cb87-4a9c-85df-26c0433afd50</v>
+        <v>ef836ab2-ae6d-420e-8900-65736d31e481</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D7" t="str">
         <v>Raa Atoll</v>
@@ -499,13 +499,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>8edf3525-64e9-4761-9eff-b05a64a7b76c</v>
+        <v>f50b1e3f-a70d-4483-a4ec-6ff1d4234f2f</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D8" t="str">
         <v>Lhaviyani Atoll</v>
@@ -513,13 +513,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>68398791-0051-406e-8506-0ca6b02a0c83</v>
+        <v>e166b76a-f3e7-413b-bc4d-477dd3200e11</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D9" t="str">
         <v>Ari Atoll</v>
@@ -527,13 +527,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>09d99f32-8cb8-4e63-aa51-1e8380cea171</v>
+        <v>3ff3b4ef-9b86-47b9-bc63-f3bb26ffc86f</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D10" t="str">
         <v>Meemu Atoll</v>
@@ -541,13 +541,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>5978af87-3103-44d8-9d83-994bc27da4ac</v>
+        <v>408b3a30-7da7-48de-a173-5a83d45f2794</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D11" t="str">
         <v>Laamu Atoll</v>
@@ -555,13 +555,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ff18591c-4ea8-4522-9edf-eb318102d4de</v>
+        <v>d0d40e87-6e2f-4d54-99de-9cf2e2c78d3f</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D12" t="str">
         <v>Gaafu Alifu Atoll</v>
@@ -569,13 +569,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>5996545e-ee01-43f7-8a07-cfccaa985f42</v>
+        <v>a4e5f5e1-7a3e-4428-8dfc-86bb3ff86450</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-02-14T10:22:02.382Z</v>
+        <v>2026-02-15T07:01:23.175Z</v>
       </c>
       <c r="D13" t="str">
         <v>Addu Atoll</v>

</xml_diff>